<commit_message>
atualizei os dados do 2Q26 da META
</commit_message>
<xml_diff>
--- a/analise_eua/tecnologia/meta/meta_indicators.xlsx
+++ b/analise_eua/tecnologia/meta/meta_indicators.xlsx
@@ -592,10 +592,10 @@
         <v>2025</v>
       </c>
       <c r="B2" t="n">
-        <v>27.5</v>
+        <v>27.48</v>
       </c>
       <c r="C2" t="n">
-        <v>27.5</v>
+        <v>27.48</v>
       </c>
       <c r="D2" t="n">
         <v>3.64</v>
@@ -610,7 +610,7 @@
         <v>7.65</v>
       </c>
       <c r="H2" t="n">
-        <v>1662675130</v>
+        <v>1661112110</v>
       </c>
       <c r="I2" t="n">
         <v>85081</v>
@@ -628,7 +628,7 @@
         <v>0.02</v>
       </c>
       <c r="N2" t="n">
-        <v>16.35</v>
+        <v>16.34</v>
       </c>
       <c r="O2" t="n">
         <v>27.83</v>
@@ -687,10 +687,10 @@
         <v>2024</v>
       </c>
       <c r="B3" t="n">
-        <v>23.7</v>
+        <v>23.68</v>
       </c>
       <c r="C3" t="n">
-        <v>23.7</v>
+        <v>23.67</v>
       </c>
       <c r="D3" t="n">
         <v>4.22</v>
@@ -702,10 +702,10 @@
         <v>37.91</v>
       </c>
       <c r="G3" t="n">
-        <v>8.09</v>
+        <v>8.08</v>
       </c>
       <c r="H3" t="n">
-        <v>1477752780</v>
+        <v>1476384420</v>
       </c>
       <c r="I3" t="n">
         <v>49769</v>
@@ -723,7 +723,7 @@
         <v>-0.15</v>
       </c>
       <c r="N3" t="n">
-        <v>17.74</v>
+        <v>17.72</v>
       </c>
       <c r="O3" t="n">
         <v>34.14</v>
@@ -782,10 +782,10 @@
         <v>2023</v>
       </c>
       <c r="B4" t="n">
-        <v>23.12</v>
+        <v>23.1</v>
       </c>
       <c r="C4" t="n">
-        <v>23.12</v>
+        <v>23.1</v>
       </c>
       <c r="D4" t="n">
         <v>4.33</v>
@@ -800,7 +800,7 @@
         <v>5.9</v>
       </c>
       <c r="H4" t="n">
-        <v>903988799.9999999</v>
+        <v>903165120</v>
       </c>
       <c r="I4" t="n">
         <v>37924</v>
@@ -818,7 +818,7 @@
         <v>-0.18</v>
       </c>
       <c r="N4" t="n">
-        <v>16.08</v>
+        <v>16.07</v>
       </c>
       <c r="O4" t="n">
         <v>25.53</v>
@@ -877,10 +877,10 @@
         <v>2022</v>
       </c>
       <c r="B5" t="n">
-        <v>13.83</v>
+        <v>13.82</v>
       </c>
       <c r="C5" t="n">
-        <v>13.84</v>
+        <v>13.82</v>
       </c>
       <c r="D5" t="n">
         <v>7.23</v>
@@ -895,7 +895,7 @@
         <v>2.55</v>
       </c>
       <c r="H5" t="n">
-        <v>320827800</v>
+        <v>320532230.0000001</v>
       </c>
       <c r="I5" t="n">
         <v>27278</v>
@@ -972,13 +972,13 @@
         <v>2021</v>
       </c>
       <c r="B6" t="n">
-        <v>23.86</v>
+        <v>23.84</v>
       </c>
       <c r="C6" t="n">
-        <v>23.85</v>
+        <v>23.83</v>
       </c>
       <c r="D6" t="n">
-        <v>4.19</v>
+        <v>4.2</v>
       </c>
       <c r="E6" t="n">
         <v>54720</v>
@@ -990,7 +990,7 @@
         <v>7.52</v>
       </c>
       <c r="H6" t="n">
-        <v>939449950.0000001</v>
+        <v>938577300</v>
       </c>
       <c r="I6" t="n">
         <v>14454</v>
@@ -1008,7 +1008,7 @@
         <v>-0.27</v>
       </c>
       <c r="N6" t="n">
-        <v>17.78</v>
+        <v>17.77</v>
       </c>
       <c r="O6" t="n">
         <v>31.53</v>
@@ -1067,10 +1067,10 @@
         <v>2020</v>
       </c>
       <c r="B7" t="n">
-        <v>26.51</v>
+        <v>26.49</v>
       </c>
       <c r="C7" t="n">
-        <v>26.52</v>
+        <v>26.5</v>
       </c>
       <c r="D7" t="n">
         <v>3.77</v>
@@ -1085,7 +1085,7 @@
         <v>6.02</v>
       </c>
       <c r="H7" t="n">
-        <v>772706529.9999999</v>
+        <v>771993779.9999999</v>
       </c>
       <c r="I7" t="n">
         <v>11177</v>
@@ -1103,7 +1103,7 @@
         <v>-0.4</v>
       </c>
       <c r="N7" t="n">
-        <v>20.83</v>
+        <v>20.81</v>
       </c>
       <c r="O7" t="n">
         <v>22.72</v>
@@ -1162,10 +1162,10 @@
         <v>2019</v>
       </c>
       <c r="B8" t="n">
-        <v>31.44</v>
+        <v>31.41</v>
       </c>
       <c r="C8" t="n">
-        <v>31.43</v>
+        <v>31.4</v>
       </c>
       <c r="D8" t="n">
         <v>3.18</v>
@@ -1180,7 +1180,7 @@
         <v>5.75</v>
       </c>
       <c r="H8" t="n">
-        <v>581217100</v>
+        <v>580674840</v>
       </c>
       <c r="I8" t="n">
         <v>10797</v>
@@ -1198,7 +1198,7 @@
         <v>-0.44</v>
       </c>
       <c r="N8" t="n">
-        <v>21.03</v>
+        <v>21.02</v>
       </c>
       <c r="O8" t="n">
         <v>18.29</v>
@@ -1257,13 +1257,13 @@
         <v>2018</v>
       </c>
       <c r="B9" t="n">
-        <v>17</v>
+        <v>16.98</v>
       </c>
       <c r="C9" t="n">
-        <v>17</v>
+        <v>16.99</v>
       </c>
       <c r="D9" t="n">
-        <v>5.88</v>
+        <v>5.89</v>
       </c>
       <c r="E9" t="n">
         <v>29228</v>
@@ -1272,10 +1272,10 @@
         <v>39.6</v>
       </c>
       <c r="G9" t="n">
-        <v>4.47</v>
+        <v>4.46</v>
       </c>
       <c r="H9" t="n">
-        <v>375902300</v>
+        <v>375555499.9999999</v>
       </c>
       <c r="I9" t="n">
         <v>14651</v>
@@ -1293,7 +1293,7 @@
         <v>-0.31</v>
       </c>
       <c r="N9" t="n">
-        <v>13.77</v>
+        <v>13.75</v>
       </c>
       <c r="O9" t="n">
         <v>26.28</v>
@@ -1352,10 +1352,10 @@
         <v>2017</v>
       </c>
       <c r="B10" t="n">
-        <v>31.88</v>
+        <v>31.85</v>
       </c>
       <c r="C10" t="n">
-        <v>31.89</v>
+        <v>31.86</v>
       </c>
       <c r="D10" t="n">
         <v>3.14</v>
@@ -1367,10 +1367,10 @@
         <v>39.2</v>
       </c>
       <c r="G10" t="n">
-        <v>6.83</v>
+        <v>6.82</v>
       </c>
       <c r="H10" t="n">
-        <v>507936090</v>
+        <v>507442920</v>
       </c>
       <c r="I10" t="n">
         <v>4644</v>
@@ -1388,7 +1388,7 @@
         <v>-0.5</v>
       </c>
       <c r="N10" t="n">
-        <v>23.46</v>
+        <v>23.44</v>
       </c>
       <c r="O10" t="n">
         <v>21.43</v>
@@ -1453,7 +1453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE17"/>
+  <dimension ref="A1:AE18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1610,94 +1610,94 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46112</v>
+        <v>46203</v>
       </c>
       <c r="B2" t="n">
-        <v>54.15</v>
+        <v>90.39</v>
       </c>
       <c r="C2" t="n">
-        <v>22.42</v>
+        <v>22.39</v>
       </c>
       <c r="D2" t="n">
-        <v>4.46</v>
+        <v>4.47</v>
       </c>
       <c r="E2" t="n">
-        <v>28871</v>
+        <v>25131</v>
       </c>
       <c r="F2" t="n">
-        <v>47.54</v>
+        <v>26.07</v>
       </c>
       <c r="G2" t="n">
-        <v>5.95</v>
+        <v>5.48</v>
       </c>
       <c r="H2" t="n">
-        <v>1449777420</v>
+        <v>1432446470</v>
       </c>
       <c r="I2" t="n">
-        <v>86769</v>
+        <v>112318</v>
       </c>
       <c r="J2" t="n">
-        <v>81180</v>
+        <v>90260</v>
       </c>
       <c r="K2" t="n">
-        <v>5589</v>
+        <v>22058</v>
       </c>
       <c r="L2" t="n">
-        <v>0.06</v>
+        <v>0.21</v>
       </c>
       <c r="M2" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
       <c r="N2" t="n">
-        <v>14.47</v>
+        <v>13.95</v>
       </c>
       <c r="O2" t="n">
-        <v>26.45</v>
+        <v>24.37</v>
       </c>
       <c r="P2" t="n">
-        <v>19.23</v>
+        <v>17.02</v>
       </c>
       <c r="Q2" t="n">
-        <v>32226</v>
+        <v>31862</v>
       </c>
       <c r="R2" t="n">
-        <v>-33678</v>
+        <v>-49653</v>
       </c>
       <c r="S2" t="n">
-        <v>-6553</v>
+        <v>15967</v>
       </c>
       <c r="T2" t="n">
-        <v>13229</v>
+        <v>1746</v>
       </c>
       <c r="U2" t="n">
-        <v>18997</v>
+        <v>30116</v>
       </c>
       <c r="V2" t="n">
-        <v>48101</v>
+        <v>62820</v>
       </c>
       <c r="W2" t="n">
-        <v>17699</v>
+        <v>21656</v>
       </c>
       <c r="X2" t="n">
-        <v>106036</v>
+        <v>130261</v>
       </c>
       <c r="Y2" t="n">
-        <v>63012</v>
+        <v>69096</v>
       </c>
       <c r="Z2" t="n">
-        <v>178.91</v>
+        <v>201.8</v>
       </c>
       <c r="AA2" t="n">
-        <v>6113</v>
+        <v>24879</v>
       </c>
       <c r="AB2" t="n">
-        <v>25666</v>
+        <v>8939</v>
       </c>
       <c r="AC2" t="n">
         <v>0.53</v>
       </c>
       <c r="AD2" t="n">
-        <v>5.03</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="AE2" t="n">
         <v>0</v>
@@ -1705,753 +1705,753 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45930</v>
+        <v>46112</v>
       </c>
       <c r="B3" t="n">
-        <v>681.1900000000001</v>
+        <v>54.1</v>
       </c>
       <c r="C3" t="n">
-        <v>34.66</v>
+        <v>22.4</v>
       </c>
       <c r="D3" t="n">
-        <v>2.88</v>
+        <v>4.46</v>
       </c>
       <c r="E3" t="n">
-        <v>25498</v>
+        <v>28871</v>
       </c>
       <c r="F3" t="n">
-        <v>5.29</v>
+        <v>47.54</v>
       </c>
       <c r="G3" t="n">
-        <v>9.51</v>
+        <v>5.94</v>
       </c>
       <c r="H3" t="n">
-        <v>1845338550</v>
+        <v>1448434400</v>
       </c>
       <c r="I3" t="n">
-        <v>51060</v>
+        <v>86769</v>
       </c>
       <c r="J3" t="n">
-        <v>44448</v>
+        <v>81180</v>
       </c>
       <c r="K3" t="n">
-        <v>6612</v>
+        <v>5589</v>
       </c>
       <c r="L3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="M3" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="N3" t="n">
-        <v>19.89</v>
+        <v>14.45</v>
       </c>
       <c r="O3" t="n">
-        <v>27.51</v>
+        <v>26.45</v>
       </c>
       <c r="P3" t="n">
-        <v>20.75</v>
+        <v>19.23</v>
       </c>
       <c r="Q3" t="n">
-        <v>29999</v>
+        <v>32226</v>
       </c>
       <c r="R3" t="n">
-        <v>-21848</v>
+        <v>-33678</v>
       </c>
       <c r="S3" t="n">
-        <v>-10047</v>
+        <v>-6553</v>
       </c>
       <c r="T3" t="n">
-        <v>11170</v>
+        <v>13229</v>
       </c>
       <c r="U3" t="n">
-        <v>18829</v>
+        <v>18997</v>
       </c>
       <c r="V3" t="n">
-        <v>39334</v>
+        <v>48101</v>
       </c>
       <c r="W3" t="n">
-        <v>15144</v>
+        <v>17699</v>
       </c>
       <c r="X3" t="n">
-        <v>90747</v>
+        <v>106036</v>
       </c>
       <c r="Y3" t="n">
-        <v>36160</v>
+        <v>63012</v>
       </c>
       <c r="Z3" t="n">
-        <v>143.6</v>
+        <v>178.91</v>
       </c>
       <c r="AA3" t="n">
-        <v>39478</v>
+        <v>6113</v>
       </c>
       <c r="AB3" t="n">
-        <v>-12129</v>
+        <v>25666</v>
       </c>
       <c r="AC3" t="n">
         <v>0.53</v>
       </c>
       <c r="AD3" t="n">
-        <v>49.1</v>
+        <v>5.03</v>
       </c>
       <c r="AE3" t="n">
-        <v>3327</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45838</v>
+        <v>45930</v>
       </c>
       <c r="B4" t="n">
-        <v>101.12</v>
+        <v>680.5599999999999</v>
       </c>
       <c r="C4" t="n">
-        <v>29.01</v>
+        <v>34.63</v>
       </c>
       <c r="D4" t="n">
-        <v>3.45</v>
+        <v>2.89</v>
       </c>
       <c r="E4" t="n">
-        <v>24783</v>
+        <v>25498</v>
       </c>
       <c r="F4" t="n">
-        <v>38.59</v>
+        <v>5.29</v>
       </c>
       <c r="G4" t="n">
-        <v>9.51</v>
+        <v>9.5</v>
       </c>
       <c r="H4" t="n">
-        <v>1854154480</v>
+        <v>1843626990</v>
       </c>
       <c r="I4" t="n">
-        <v>49560</v>
+        <v>51060</v>
       </c>
       <c r="J4" t="n">
-        <v>47071</v>
+        <v>44448</v>
       </c>
       <c r="K4" t="n">
-        <v>2489</v>
+        <v>6612</v>
       </c>
       <c r="L4" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="M4" t="n">
         <v>0.03</v>
       </c>
-      <c r="M4" t="n">
-        <v>0.01</v>
-      </c>
       <c r="N4" t="n">
-        <v>21.56</v>
+        <v>19.87</v>
       </c>
       <c r="O4" t="n">
-        <v>32.88</v>
+        <v>27.51</v>
       </c>
       <c r="P4" t="n">
-        <v>25.54</v>
+        <v>20.75</v>
       </c>
       <c r="Q4" t="n">
-        <v>25561</v>
+        <v>29999</v>
       </c>
       <c r="R4" t="n">
-        <v>-25958</v>
+        <v>-21848</v>
       </c>
       <c r="S4" t="n">
-        <v>-15977</v>
+        <v>-10047</v>
       </c>
       <c r="T4" t="n">
-        <v>9023</v>
+        <v>11170</v>
       </c>
       <c r="U4" t="n">
-        <v>16538</v>
+        <v>18829</v>
       </c>
       <c r="V4" t="n">
-        <v>30004</v>
+        <v>39334</v>
       </c>
       <c r="W4" t="n">
-        <v>12942</v>
+        <v>15144</v>
       </c>
       <c r="X4" t="n">
-        <v>76810</v>
+        <v>90747</v>
       </c>
       <c r="Y4" t="n">
-        <v>36308</v>
+        <v>36160</v>
       </c>
       <c r="Z4" t="n">
-        <v>126.33</v>
+        <v>143.6</v>
       </c>
       <c r="AA4" t="n">
-        <v>39967</v>
+        <v>39478</v>
       </c>
       <c r="AB4" t="n">
-        <v>30552</v>
+        <v>-12129</v>
       </c>
       <c r="AC4" t="n">
         <v>0.53</v>
       </c>
       <c r="AD4" t="n">
-        <v>7.24</v>
+        <v>49.1</v>
       </c>
       <c r="AE4" t="n">
-        <v>10167</v>
+        <v>3327</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45747</v>
+        <v>45838</v>
       </c>
       <c r="B5" t="n">
-        <v>87.23</v>
+        <v>101.02</v>
       </c>
       <c r="C5" t="n">
-        <v>25.02</v>
+        <v>28.99</v>
       </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>3.45</v>
       </c>
       <c r="E5" t="n">
-        <v>21455</v>
+        <v>24783</v>
       </c>
       <c r="F5" t="n">
-        <v>39.33</v>
+        <v>38.59</v>
       </c>
       <c r="G5" t="n">
-        <v>7.85</v>
+        <v>9.5</v>
       </c>
       <c r="H5" t="n">
-        <v>1451938390</v>
+        <v>1852442240</v>
       </c>
       <c r="I5" t="n">
-        <v>49519</v>
+        <v>49560</v>
       </c>
       <c r="J5" t="n">
-        <v>70230</v>
+        <v>47071</v>
       </c>
       <c r="K5" t="n">
-        <v>-20711</v>
+        <v>2489</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.26</v>
+        <v>0.03</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.11</v>
+        <v>0.01</v>
       </c>
       <c r="N5" t="n">
-        <v>18.76</v>
+        <v>21.54</v>
       </c>
       <c r="O5" t="n">
-        <v>31.44</v>
+        <v>32.88</v>
       </c>
       <c r="P5" t="n">
-        <v>23.98</v>
+        <v>25.54</v>
       </c>
       <c r="Q5" t="n">
-        <v>24026</v>
+        <v>25561</v>
       </c>
       <c r="R5" t="n">
-        <v>-20010</v>
+        <v>-25958</v>
       </c>
       <c r="S5" t="n">
-        <v>-19495</v>
+        <v>-15977</v>
       </c>
       <c r="T5" t="n">
-        <v>11085</v>
+        <v>9023</v>
       </c>
       <c r="U5" t="n">
-        <v>12941</v>
+        <v>16538</v>
       </c>
       <c r="V5" t="n">
-        <v>20834</v>
+        <v>30004</v>
       </c>
       <c r="W5" t="n">
-        <v>12150</v>
+        <v>12942</v>
       </c>
       <c r="X5" t="n">
-        <v>64676</v>
+        <v>76810</v>
       </c>
       <c r="Y5" t="n">
-        <v>56337</v>
+        <v>36308</v>
       </c>
       <c r="Z5" t="n">
-        <v>115.77</v>
+        <v>126.33</v>
       </c>
       <c r="AA5" t="n">
-        <v>45021</v>
+        <v>39967</v>
       </c>
       <c r="AB5" t="n">
-        <v>36292</v>
+        <v>30552</v>
       </c>
       <c r="AC5" t="n">
         <v>0.53</v>
       </c>
       <c r="AD5" t="n">
-        <v>7.98</v>
+        <v>7.24</v>
       </c>
       <c r="AE5" t="n">
-        <v>12754</v>
+        <v>10167</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45565</v>
+        <v>45747</v>
       </c>
       <c r="B6" t="n">
-        <v>91.84</v>
+        <v>87.15000000000001</v>
       </c>
       <c r="C6" t="n">
-        <v>27.3</v>
+        <v>25</v>
       </c>
       <c r="D6" t="n">
-        <v>3.66</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>21377</v>
+        <v>21455</v>
       </c>
       <c r="F6" t="n">
-        <v>38.65</v>
+        <v>39.33</v>
       </c>
       <c r="G6" t="n">
-        <v>8.76</v>
+        <v>7.84</v>
       </c>
       <c r="H6" t="n">
-        <v>1440746010</v>
+        <v>1450599080</v>
       </c>
       <c r="I6" t="n">
-        <v>49047</v>
+        <v>49519</v>
       </c>
       <c r="J6" t="n">
-        <v>70900</v>
+        <v>70230</v>
       </c>
       <c r="K6" t="n">
-        <v>-21853</v>
+        <v>-20711</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.3</v>
+        <v>-0.26</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.13</v>
+        <v>-0.11</v>
       </c>
       <c r="N6" t="n">
-        <v>19.86</v>
+        <v>18.74</v>
       </c>
       <c r="O6" t="n">
-        <v>32.28</v>
+        <v>31.44</v>
       </c>
       <c r="P6" t="n">
-        <v>24.22</v>
+        <v>23.98</v>
       </c>
       <c r="Q6" t="n">
-        <v>24724</v>
+        <v>24026</v>
       </c>
       <c r="R6" t="n">
-        <v>-8620</v>
+        <v>-20010</v>
       </c>
       <c r="S6" t="n">
-        <v>-4371</v>
+        <v>-19495</v>
       </c>
       <c r="T6" t="n">
-        <v>16466</v>
+        <v>11085</v>
       </c>
       <c r="U6" t="n">
-        <v>8258</v>
+        <v>12941</v>
       </c>
       <c r="V6" t="n">
-        <v>15477</v>
+        <v>20834</v>
       </c>
       <c r="W6" t="n">
-        <v>11177</v>
+        <v>12150</v>
       </c>
       <c r="X6" t="n">
-        <v>56410</v>
+        <v>64676</v>
       </c>
       <c r="Y6" t="n">
-        <v>57737</v>
+        <v>56337</v>
       </c>
       <c r="Z6" t="n">
-        <v>107.56</v>
+        <v>115.77</v>
       </c>
       <c r="AA6" t="n">
-        <v>46997</v>
+        <v>45021</v>
       </c>
       <c r="AB6" t="n">
-        <v>37892</v>
+        <v>36292</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="AD6" t="n">
-        <v>8.050000000000001</v>
+        <v>7.98</v>
       </c>
       <c r="AE6" t="n">
-        <v>8818</v>
+        <v>12754</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45473</v>
+        <v>45565</v>
       </c>
       <c r="B7" t="n">
-        <v>94.34</v>
+        <v>91.75</v>
       </c>
       <c r="C7" t="n">
-        <v>28.32</v>
+        <v>27.27</v>
       </c>
       <c r="D7" t="n">
-        <v>3.53</v>
+        <v>3.67</v>
       </c>
       <c r="E7" t="n">
-        <v>18484</v>
+        <v>21377</v>
       </c>
       <c r="F7" t="n">
-        <v>34.46</v>
+        <v>38.65</v>
       </c>
       <c r="G7" t="n">
-        <v>8.1</v>
+        <v>8.75</v>
       </c>
       <c r="H7" t="n">
-        <v>1270344880</v>
+        <v>1439430930</v>
       </c>
       <c r="I7" t="n">
-        <v>37991</v>
+        <v>49047</v>
       </c>
       <c r="J7" t="n">
-        <v>58080</v>
+        <v>70900</v>
       </c>
       <c r="K7" t="n">
-        <v>-20089</v>
+        <v>-21853</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.31</v>
+        <v>-0.3</v>
       </c>
       <c r="M7" t="n">
         <v>-0.13</v>
       </c>
       <c r="N7" t="n">
-        <v>20.07</v>
+        <v>19.84</v>
       </c>
       <c r="O7" t="n">
-        <v>28.84</v>
+        <v>32.28</v>
       </c>
       <c r="P7" t="n">
-        <v>22.8</v>
+        <v>24.22</v>
       </c>
       <c r="Q7" t="n">
-        <v>19370</v>
+        <v>24724</v>
       </c>
       <c r="R7" t="n">
-        <v>-8298</v>
+        <v>-8620</v>
       </c>
       <c r="S7" t="n">
-        <v>-11178</v>
+        <v>-4371</v>
       </c>
       <c r="T7" t="n">
-        <v>11197</v>
+        <v>16466</v>
       </c>
       <c r="U7" t="n">
-        <v>8173</v>
+        <v>8258</v>
       </c>
       <c r="V7" t="n">
-        <v>14839</v>
+        <v>15477</v>
       </c>
       <c r="W7" t="n">
-        <v>10537</v>
+        <v>11177</v>
       </c>
       <c r="X7" t="n">
-        <v>53939</v>
+        <v>56410</v>
       </c>
       <c r="Y7" t="n">
-        <v>49427</v>
+        <v>57737</v>
       </c>
       <c r="Z7" t="n">
-        <v>126.83</v>
+        <v>107.56</v>
       </c>
       <c r="AA7" t="n">
-        <v>35337</v>
+        <v>46997</v>
       </c>
       <c r="AB7" t="n">
-        <v>28955</v>
+        <v>37892</v>
       </c>
       <c r="AC7" t="n">
         <v>0.5</v>
       </c>
       <c r="AD7" t="n">
-        <v>9.4</v>
+        <v>8.050000000000001</v>
       </c>
       <c r="AE7" t="n">
-        <v>6299</v>
+        <v>8818</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45382</v>
+        <v>45473</v>
       </c>
       <c r="B8" t="n">
-        <v>99.23999999999999</v>
+        <v>94.26000000000001</v>
       </c>
       <c r="C8" t="n">
-        <v>33.03</v>
+        <v>28.3</v>
       </c>
       <c r="D8" t="n">
-        <v>3.03</v>
+        <v>3.53</v>
       </c>
       <c r="E8" t="n">
-        <v>17192</v>
+        <v>18484</v>
       </c>
       <c r="F8" t="n">
-        <v>33.93</v>
+        <v>34.46</v>
       </c>
       <c r="G8" t="n">
-        <v>8.210000000000001</v>
+        <v>8.1</v>
       </c>
       <c r="H8" t="n">
-        <v>1227478950</v>
+        <v>1269179240</v>
       </c>
       <c r="I8" t="n">
-        <v>37633</v>
+        <v>37991</v>
       </c>
       <c r="J8" t="n">
-        <v>58120</v>
+        <v>58080</v>
       </c>
       <c r="K8" t="n">
-        <v>-20487</v>
+        <v>-20089</v>
       </c>
       <c r="L8" t="n">
-        <v>-0.37</v>
+        <v>-0.31</v>
       </c>
       <c r="M8" t="n">
-        <v>-0.14</v>
+        <v>-0.13</v>
       </c>
       <c r="N8" t="n">
-        <v>22.46</v>
+        <v>20.05</v>
       </c>
       <c r="O8" t="n">
-        <v>25.04</v>
+        <v>28.84</v>
       </c>
       <c r="P8" t="n">
-        <v>19.68</v>
+        <v>22.8</v>
       </c>
       <c r="Q8" t="n">
-        <v>19246</v>
+        <v>19370</v>
       </c>
       <c r="R8" t="n">
-        <v>-8734</v>
+        <v>-8298</v>
       </c>
       <c r="S8" t="n">
-        <v>-19767</v>
+        <v>-11178</v>
       </c>
       <c r="T8" t="n">
-        <v>12846</v>
+        <v>11197</v>
       </c>
       <c r="U8" t="n">
-        <v>6400</v>
+        <v>8173</v>
       </c>
       <c r="V8" t="n">
-        <v>14621</v>
+        <v>14839</v>
       </c>
       <c r="W8" t="n">
-        <v>9978</v>
+        <v>10537</v>
       </c>
       <c r="X8" t="n">
-        <v>52565</v>
+        <v>53939</v>
       </c>
       <c r="Y8" t="n">
-        <v>47229</v>
+        <v>49427</v>
       </c>
       <c r="Z8" t="n">
-        <v>143.35</v>
+        <v>126.83</v>
       </c>
       <c r="AA8" t="n">
-        <v>29984</v>
+        <v>35337</v>
       </c>
       <c r="AB8" t="n">
-        <v>23680</v>
+        <v>28955</v>
       </c>
       <c r="AC8" t="n">
         <v>0.5</v>
       </c>
       <c r="AD8" t="n">
-        <v>10.29</v>
+        <v>9.4</v>
       </c>
       <c r="AE8" t="n">
-        <v>15008</v>
+        <v>6299</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45199</v>
+        <v>45382</v>
       </c>
       <c r="B9" t="n">
-        <v>66.23999999999999</v>
+        <v>99.15000000000001</v>
       </c>
       <c r="C9" t="n">
-        <v>26.17</v>
+        <v>33</v>
       </c>
       <c r="D9" t="n">
-        <v>3.82</v>
+        <v>3.03</v>
       </c>
       <c r="E9" t="n">
-        <v>16607</v>
+        <v>17192</v>
       </c>
       <c r="F9" t="n">
-        <v>33.92</v>
+        <v>33.93</v>
       </c>
       <c r="G9" t="n">
-        <v>5.37</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>767313120</v>
+        <v>1226333700</v>
       </c>
       <c r="I9" t="n">
-        <v>36217</v>
+        <v>37633</v>
       </c>
       <c r="J9" t="n">
-        <v>61123</v>
+        <v>58120</v>
       </c>
       <c r="K9" t="n">
-        <v>-24906</v>
+        <v>-20487</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.54</v>
+        <v>-0.37</v>
       </c>
       <c r="M9" t="n">
-        <v>-0.17</v>
+        <v>-0.14</v>
       </c>
       <c r="N9" t="n">
-        <v>17.14</v>
+        <v>22.44</v>
       </c>
       <c r="O9" t="n">
-        <v>20.63</v>
+        <v>25.04</v>
       </c>
       <c r="P9" t="n">
-        <v>16.37</v>
+        <v>19.68</v>
       </c>
       <c r="Q9" t="n">
-        <v>20402</v>
+        <v>19246</v>
       </c>
       <c r="R9" t="n">
-        <v>-6077</v>
+        <v>-8734</v>
       </c>
       <c r="S9" t="n">
-        <v>-5875</v>
+        <v>-19767</v>
       </c>
       <c r="T9" t="n">
-        <v>13859</v>
+        <v>12846</v>
       </c>
       <c r="U9" t="n">
-        <v>6543</v>
+        <v>6400</v>
       </c>
       <c r="V9" t="n">
-        <v>18795</v>
+        <v>14621</v>
       </c>
       <c r="W9" t="n">
-        <v>9241</v>
+        <v>9978</v>
       </c>
       <c r="X9" t="n">
-        <v>55931</v>
+        <v>52565</v>
       </c>
       <c r="Y9" t="n">
-        <v>47847</v>
+        <v>47229</v>
       </c>
       <c r="Z9" t="n">
-        <v>183.85</v>
+        <v>143.35</v>
       </c>
       <c r="AA9" t="n">
-        <v>30187</v>
+        <v>29984</v>
       </c>
       <c r="AB9" t="n">
-        <v>13018</v>
+        <v>23680</v>
       </c>
       <c r="AC9" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="AD9" t="n">
-        <v>0</v>
+        <v>10.29</v>
       </c>
       <c r="AE9" t="n">
-        <v>3569</v>
+        <v>15008</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45107</v>
+        <v>45199</v>
       </c>
       <c r="B10" t="n">
-        <v>93.89</v>
+        <v>66.18000000000001</v>
       </c>
       <c r="C10" t="n">
-        <v>30.45</v>
+        <v>26.15</v>
       </c>
       <c r="D10" t="n">
-        <v>3.28</v>
+        <v>3.82</v>
       </c>
       <c r="E10" t="n">
-        <v>12015</v>
+        <v>16607</v>
       </c>
       <c r="F10" t="n">
-        <v>24.34</v>
+        <v>33.92</v>
       </c>
       <c r="G10" t="n">
-        <v>5.46</v>
+        <v>5.37</v>
       </c>
       <c r="H10" t="n">
-        <v>731238000</v>
+        <v>766617600.0000001</v>
       </c>
       <c r="I10" t="n">
-        <v>36218</v>
+        <v>36217</v>
       </c>
       <c r="J10" t="n">
-        <v>53446</v>
+        <v>61123</v>
       </c>
       <c r="K10" t="n">
-        <v>-17228</v>
+        <v>-24906</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.43</v>
+        <v>-0.54</v>
       </c>
       <c r="M10" t="n">
-        <v>-0.13</v>
+        <v>-0.17</v>
       </c>
       <c r="N10" t="n">
-        <v>18.74</v>
+        <v>17.13</v>
       </c>
       <c r="O10" t="n">
-        <v>18.34</v>
+        <v>20.63</v>
       </c>
       <c r="P10" t="n">
-        <v>14.6</v>
+        <v>16.37</v>
       </c>
       <c r="Q10" t="n">
-        <v>17309</v>
+        <v>20402</v>
       </c>
       <c r="R10" t="n">
-        <v>-5203</v>
+        <v>-6077</v>
       </c>
       <c r="S10" t="n">
-        <v>5292</v>
+        <v>-5875</v>
       </c>
       <c r="T10" t="n">
-        <v>11093</v>
+        <v>13859</v>
       </c>
       <c r="U10" t="n">
-        <v>6216</v>
+        <v>6543</v>
       </c>
       <c r="V10" t="n">
-        <v>20704</v>
+        <v>18795</v>
       </c>
       <c r="W10" t="n">
-        <v>9344</v>
+        <v>9241</v>
       </c>
       <c r="X10" t="n">
-        <v>57289</v>
+        <v>55931</v>
       </c>
       <c r="Y10" t="n">
-        <v>39639</v>
+        <v>47847</v>
       </c>
       <c r="Z10" t="n">
-        <v>220.37</v>
+        <v>183.85</v>
       </c>
       <c r="AA10" t="n">
-        <v>23895</v>
+        <v>30187</v>
       </c>
       <c r="AB10" t="n">
-        <v>7485</v>
+        <v>13018</v>
       </c>
       <c r="AC10" t="n">
         <v>0</v>
@@ -2460,93 +2460,93 @@
         <v>0</v>
       </c>
       <c r="AE10" t="n">
-        <v>898</v>
+        <v>3569</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>45016</v>
+        <v>45107</v>
       </c>
       <c r="B11" t="n">
-        <v>95.29000000000001</v>
+        <v>93.8</v>
       </c>
       <c r="C11" t="n">
-        <v>23.21</v>
+        <v>30.43</v>
       </c>
       <c r="D11" t="n">
-        <v>4.31</v>
+        <v>3.29</v>
       </c>
       <c r="E11" t="n">
-        <v>9751</v>
+        <v>12015</v>
       </c>
       <c r="F11" t="n">
-        <v>19.93</v>
+        <v>24.34</v>
       </c>
       <c r="G11" t="n">
-        <v>4.36</v>
+        <v>5.45</v>
       </c>
       <c r="H11" t="n">
-        <v>544020230</v>
+        <v>730544640</v>
       </c>
       <c r="I11" t="n">
-        <v>27575</v>
+        <v>36218</v>
       </c>
       <c r="J11" t="n">
-        <v>37439</v>
+        <v>53446</v>
       </c>
       <c r="K11" t="n">
-        <v>-9864</v>
+        <v>-17228</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.26</v>
+        <v>-0.43</v>
       </c>
       <c r="M11" t="n">
-        <v>-0.08</v>
+        <v>-0.13</v>
       </c>
       <c r="N11" t="n">
-        <v>14.35</v>
+        <v>18.72</v>
       </c>
       <c r="O11" t="n">
-        <v>19.44</v>
+        <v>18.34</v>
       </c>
       <c r="P11" t="n">
-        <v>15.79</v>
+        <v>14.6</v>
       </c>
       <c r="Q11" t="n">
-        <v>13998</v>
+        <v>17309</v>
       </c>
       <c r="R11" t="n">
-        <v>-6743</v>
+        <v>-5203</v>
       </c>
       <c r="S11" t="n">
-        <v>-10516</v>
+        <v>5292</v>
       </c>
       <c r="T11" t="n">
-        <v>7156</v>
+        <v>11093</v>
       </c>
       <c r="U11" t="n">
-        <v>6842</v>
+        <v>6216</v>
       </c>
       <c r="V11" t="n">
-        <v>20396</v>
+        <v>20704</v>
       </c>
       <c r="W11" t="n">
-        <v>9381</v>
+        <v>9344</v>
       </c>
       <c r="X11" t="n">
-        <v>55344</v>
+        <v>57289</v>
       </c>
       <c r="Y11" t="n">
-        <v>27102</v>
+        <v>39639</v>
       </c>
       <c r="Z11" t="n">
-        <v>220.99</v>
+        <v>220.37</v>
       </c>
       <c r="AA11" t="n">
-        <v>15093</v>
+        <v>23895</v>
       </c>
       <c r="AB11" t="n">
-        <v>5057</v>
+        <v>7485</v>
       </c>
       <c r="AC11" t="n">
         <v>0</v>
@@ -2555,93 +2555,93 @@
         <v>0</v>
       </c>
       <c r="AE11" t="n">
-        <v>9365</v>
+        <v>898</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>44834</v>
+        <v>45016</v>
       </c>
       <c r="B12" t="n">
-        <v>82.15000000000001</v>
+        <v>95.20999999999999</v>
       </c>
       <c r="C12" t="n">
-        <v>13.3</v>
+        <v>23.19</v>
       </c>
       <c r="D12" t="n">
-        <v>7.52</v>
+        <v>4.31</v>
       </c>
       <c r="E12" t="n">
-        <v>7839</v>
+        <v>9751</v>
       </c>
       <c r="F12" t="n">
-        <v>15.86</v>
+        <v>19.93</v>
       </c>
       <c r="G12" t="n">
-        <v>2.91</v>
+        <v>4.36</v>
       </c>
       <c r="H12" t="n">
-        <v>361050840</v>
+        <v>543528700</v>
       </c>
       <c r="I12" t="n">
-        <v>25900</v>
+        <v>27575</v>
       </c>
       <c r="J12" t="n">
-        <v>41776</v>
+        <v>37439</v>
       </c>
       <c r="K12" t="n">
-        <v>-15876</v>
+        <v>-9864</v>
       </c>
       <c r="L12" t="n">
-        <v>-0.38</v>
+        <v>-0.26</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.13</v>
+        <v>-0.08</v>
       </c>
       <c r="N12" t="n">
-        <v>9.130000000000001</v>
+        <v>14.33</v>
       </c>
       <c r="O12" t="n">
-        <v>22.35</v>
+        <v>19.44</v>
       </c>
       <c r="P12" t="n">
-        <v>18.32</v>
+        <v>15.79</v>
       </c>
       <c r="Q12" t="n">
-        <v>9692</v>
+        <v>13998</v>
       </c>
       <c r="R12" t="n">
-        <v>-9701</v>
+        <v>-6743</v>
       </c>
       <c r="S12" t="n">
-        <v>2147</v>
+        <v>-10516</v>
       </c>
       <c r="T12" t="n">
-        <v>317</v>
+        <v>7156</v>
       </c>
       <c r="U12" t="n">
-        <v>9375</v>
+        <v>6842</v>
       </c>
       <c r="V12" t="n">
-        <v>18397</v>
+        <v>20396</v>
       </c>
       <c r="W12" t="n">
-        <v>9170</v>
+        <v>9381</v>
       </c>
       <c r="X12" t="n">
-        <v>50280</v>
+        <v>55344</v>
       </c>
       <c r="Y12" t="n">
-        <v>35628</v>
+        <v>27102</v>
       </c>
       <c r="Z12" t="n">
-        <v>184.98</v>
+        <v>220.99</v>
       </c>
       <c r="AA12" t="n">
-        <v>17876</v>
+        <v>15093</v>
       </c>
       <c r="AB12" t="n">
-        <v>7046</v>
+        <v>5057</v>
       </c>
       <c r="AC12" t="n">
         <v>0</v>
@@ -2650,93 +2650,93 @@
         <v>0</v>
       </c>
       <c r="AE12" t="n">
-        <v>6354</v>
+        <v>9365</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>44742</v>
+        <v>44834</v>
       </c>
       <c r="B13" t="n">
-        <v>64.69</v>
+        <v>82.08</v>
       </c>
       <c r="C13" t="n">
-        <v>13.17</v>
+        <v>13.29</v>
       </c>
       <c r="D13" t="n">
-        <v>7.59</v>
+        <v>7.52</v>
       </c>
       <c r="E13" t="n">
-        <v>10337</v>
+        <v>7839</v>
       </c>
       <c r="F13" t="n">
-        <v>23.2</v>
+        <v>15.86</v>
       </c>
       <c r="G13" t="n">
-        <v>3.44</v>
+        <v>2.91</v>
       </c>
       <c r="H13" t="n">
-        <v>432612960</v>
+        <v>360729000</v>
       </c>
       <c r="I13" t="n">
-        <v>16067</v>
+        <v>25900</v>
       </c>
       <c r="J13" t="n">
-        <v>40489</v>
+        <v>41776</v>
       </c>
       <c r="K13" t="n">
-        <v>-24422</v>
+        <v>-15876</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.51</v>
+        <v>-0.38</v>
       </c>
       <c r="M13" t="n">
-        <v>-0.19</v>
+        <v>-0.13</v>
       </c>
       <c r="N13" t="n">
-        <v>9.56</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="O13" t="n">
-        <v>26.83</v>
+        <v>22.35</v>
       </c>
       <c r="P13" t="n">
-        <v>23.44</v>
+        <v>18.32</v>
       </c>
       <c r="Q13" t="n">
-        <v>12196</v>
+        <v>9692</v>
       </c>
       <c r="R13" t="n">
-        <v>-6959</v>
+        <v>-9701</v>
       </c>
       <c r="S13" t="n">
-        <v>-6563</v>
+        <v>2147</v>
       </c>
       <c r="T13" t="n">
-        <v>4624</v>
+        <v>317</v>
       </c>
       <c r="U13" t="n">
-        <v>7572</v>
+        <v>9375</v>
       </c>
       <c r="V13" t="n">
-        <v>13823</v>
+        <v>18397</v>
       </c>
       <c r="W13" t="n">
-        <v>8690</v>
+        <v>9170</v>
       </c>
       <c r="X13" t="n">
-        <v>42632</v>
+        <v>50280</v>
       </c>
       <c r="Y13" t="n">
-        <v>33770</v>
+        <v>35628</v>
       </c>
       <c r="Z13" t="n">
-        <v>128.57</v>
+        <v>184.98</v>
       </c>
       <c r="AA13" t="n">
-        <v>19005</v>
+        <v>17876</v>
       </c>
       <c r="AB13" t="n">
-        <v>18478</v>
+        <v>7046</v>
       </c>
       <c r="AC13" t="n">
         <v>0</v>
@@ -2745,93 +2745,93 @@
         <v>0</v>
       </c>
       <c r="AE13" t="n">
-        <v>5233</v>
+        <v>6354</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>44651</v>
+        <v>44742</v>
       </c>
       <c r="B14" t="n">
-        <v>80.54000000000001</v>
+        <v>64.64</v>
       </c>
       <c r="C14" t="n">
-        <v>16.95</v>
+        <v>13.16</v>
       </c>
       <c r="D14" t="n">
-        <v>5.9</v>
+        <v>7.6</v>
       </c>
       <c r="E14" t="n">
-        <v>10680</v>
+        <v>10337</v>
       </c>
       <c r="F14" t="n">
-        <v>26.75</v>
+        <v>23.2</v>
       </c>
       <c r="G14" t="n">
-        <v>4.88</v>
+        <v>3.44</v>
       </c>
       <c r="H14" t="n">
-        <v>601216750</v>
+        <v>432234399.9999999</v>
       </c>
       <c r="I14" t="n">
-        <v>14053</v>
+        <v>16067</v>
       </c>
       <c r="J14" t="n">
-        <v>43890</v>
+        <v>40489</v>
       </c>
       <c r="K14" t="n">
-        <v>-29837</v>
+        <v>-24422</v>
       </c>
       <c r="L14" t="n">
-        <v>-0.59</v>
+        <v>-0.51</v>
       </c>
       <c r="M14" t="n">
-        <v>-0.24</v>
+        <v>-0.19</v>
       </c>
       <c r="N14" t="n">
-        <v>12.42</v>
+        <v>9.56</v>
       </c>
       <c r="O14" t="n">
-        <v>29.66</v>
+        <v>26.83</v>
       </c>
       <c r="P14" t="n">
-        <v>26.04</v>
+        <v>23.44</v>
       </c>
       <c r="Q14" t="n">
-        <v>14076</v>
+        <v>12196</v>
       </c>
       <c r="R14" t="n">
-        <v>-4779</v>
+        <v>-6959</v>
       </c>
       <c r="S14" t="n">
-        <v>-10660</v>
+        <v>-6563</v>
       </c>
       <c r="T14" t="n">
-        <v>8635</v>
+        <v>4624</v>
       </c>
       <c r="U14" t="n">
-        <v>5441</v>
+        <v>7572</v>
       </c>
       <c r="V14" t="n">
-        <v>10530</v>
+        <v>13823</v>
       </c>
       <c r="W14" t="n">
-        <v>7707</v>
+        <v>8690</v>
       </c>
       <c r="X14" t="n">
-        <v>35846</v>
+        <v>42632</v>
       </c>
       <c r="Y14" t="n">
-        <v>38179</v>
+        <v>33770</v>
       </c>
       <c r="Z14" t="n">
-        <v>93.73</v>
+        <v>128.57</v>
       </c>
       <c r="AA14" t="n">
-        <v>27617</v>
+        <v>19005</v>
       </c>
       <c r="AB14" t="n">
-        <v>27581</v>
+        <v>18478</v>
       </c>
       <c r="AC14" t="n">
         <v>0</v>
@@ -2840,93 +2840,93 @@
         <v>0</v>
       </c>
       <c r="AE14" t="n">
-        <v>9506</v>
+        <v>5233</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>44469</v>
+        <v>44651</v>
       </c>
       <c r="B15" t="n">
-        <v>103.07</v>
+        <v>80.45999999999999</v>
       </c>
       <c r="C15" t="n">
-        <v>25.84</v>
+        <v>16.93</v>
       </c>
       <c r="D15" t="n">
-        <v>3.87</v>
+        <v>5.91</v>
       </c>
       <c r="E15" t="n">
-        <v>12418</v>
+        <v>10680</v>
       </c>
       <c r="F15" t="n">
-        <v>31.69</v>
+        <v>26.75</v>
       </c>
       <c r="G15" t="n">
-        <v>7.11</v>
+        <v>4.87</v>
       </c>
       <c r="H15" t="n">
-        <v>947614500</v>
+        <v>600644500</v>
       </c>
       <c r="I15" t="n">
-        <v>12640</v>
+        <v>14053</v>
       </c>
       <c r="J15" t="n">
-        <v>58075</v>
+        <v>43890</v>
       </c>
       <c r="K15" t="n">
-        <v>-45435</v>
+        <v>-29837</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.91</v>
+        <v>-0.59</v>
       </c>
       <c r="M15" t="n">
-        <v>-0.34</v>
+        <v>-0.24</v>
       </c>
       <c r="N15" t="n">
-        <v>19.92</v>
+        <v>12.41</v>
       </c>
       <c r="O15" t="n">
-        <v>27.69</v>
+        <v>29.66</v>
       </c>
       <c r="P15" t="n">
-        <v>24.95</v>
+        <v>26.04</v>
       </c>
       <c r="Q15" t="n">
-        <v>14090</v>
+        <v>14076</v>
       </c>
       <c r="R15" t="n">
-        <v>-330</v>
+        <v>-4779</v>
       </c>
       <c r="S15" t="n">
-        <v>-15252</v>
+        <v>-10660</v>
       </c>
       <c r="T15" t="n">
-        <v>9776</v>
+        <v>8635</v>
       </c>
       <c r="U15" t="n">
-        <v>4314</v>
+        <v>5441</v>
       </c>
       <c r="V15" t="n">
-        <v>9236</v>
+        <v>10530</v>
       </c>
       <c r="W15" t="n">
-        <v>6316</v>
+        <v>7707</v>
       </c>
       <c r="X15" t="n">
-        <v>31608</v>
+        <v>35846</v>
       </c>
       <c r="Y15" t="n">
-        <v>57609</v>
+        <v>38179</v>
       </c>
       <c r="Z15" t="n">
-        <v>85.27</v>
+        <v>93.73</v>
       </c>
       <c r="AA15" t="n">
-        <v>27550</v>
+        <v>27617</v>
       </c>
       <c r="AB15" t="n">
-        <v>28044</v>
+        <v>27581</v>
       </c>
       <c r="AC15" t="n">
         <v>0</v>
@@ -2935,93 +2935,93 @@
         <v>0</v>
       </c>
       <c r="AE15" t="n">
-        <v>13458</v>
+        <v>9506</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>44377</v>
+        <v>44469</v>
       </c>
       <c r="B16" t="n">
-        <v>94.06999999999999</v>
+        <v>102.97</v>
       </c>
       <c r="C16" t="n">
-        <v>29.79</v>
+        <v>25.82</v>
       </c>
       <c r="D16" t="n">
-        <v>3.36</v>
+        <v>3.87</v>
       </c>
       <c r="E16" t="n">
-        <v>14353</v>
+        <v>12418</v>
       </c>
       <c r="F16" t="n">
-        <v>35.75</v>
+        <v>31.69</v>
       </c>
       <c r="G16" t="n">
-        <v>7.07</v>
+        <v>7.1</v>
       </c>
       <c r="H16" t="n">
-        <v>977730000</v>
+        <v>946742160</v>
       </c>
       <c r="I16" t="n">
-        <v>12007</v>
+        <v>12640</v>
       </c>
       <c r="J16" t="n">
-        <v>64080</v>
+        <v>58075</v>
       </c>
       <c r="K16" t="n">
-        <v>-52073</v>
+        <v>-45435</v>
       </c>
       <c r="L16" t="n">
-        <v>-1.15</v>
+        <v>-0.91</v>
       </c>
       <c r="M16" t="n">
-        <v>-0.38</v>
+        <v>-0.34</v>
       </c>
       <c r="N16" t="n">
-        <v>22.83</v>
+        <v>19.9</v>
       </c>
       <c r="O16" t="n">
-        <v>23.81</v>
+        <v>27.69</v>
       </c>
       <c r="P16" t="n">
-        <v>21.56</v>
+        <v>24.95</v>
       </c>
       <c r="Q16" t="n">
-        <v>13247</v>
+        <v>14090</v>
       </c>
       <c r="R16" t="n">
-        <v>-8195</v>
+        <v>-330</v>
       </c>
       <c r="S16" t="n">
-        <v>-8549</v>
+        <v>-15252</v>
       </c>
       <c r="T16" t="n">
-        <v>8635</v>
+        <v>9776</v>
       </c>
       <c r="U16" t="n">
-        <v>4612</v>
+        <v>4314</v>
       </c>
       <c r="V16" t="n">
-        <v>8468</v>
+        <v>9236</v>
       </c>
       <c r="W16" t="n">
-        <v>6096</v>
+        <v>6316</v>
       </c>
       <c r="X16" t="n">
-        <v>28986</v>
+        <v>31608</v>
       </c>
       <c r="Y16" t="n">
-        <v>65823</v>
+        <v>57609</v>
       </c>
       <c r="Z16" t="n">
-        <v>94.45999999999999</v>
+        <v>85.27</v>
       </c>
       <c r="AA16" t="n">
-        <v>22272</v>
+        <v>27550</v>
       </c>
       <c r="AB16" t="n">
-        <v>21285</v>
+        <v>28044</v>
       </c>
       <c r="AC16" t="n">
         <v>0</v>
@@ -3030,101 +3030,196 @@
         <v>0</v>
       </c>
       <c r="AE16" t="n">
-        <v>7079</v>
+        <v>13458</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
+        <v>44377</v>
+      </c>
+      <c r="B17" t="n">
+        <v>93.98</v>
+      </c>
+      <c r="C17" t="n">
+        <v>29.77</v>
+      </c>
+      <c r="D17" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="E17" t="n">
+        <v>14353</v>
+      </c>
+      <c r="F17" t="n">
+        <v>35.75</v>
+      </c>
+      <c r="G17" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="H17" t="n">
+        <v>976823120</v>
+      </c>
+      <c r="I17" t="n">
+        <v>12007</v>
+      </c>
+      <c r="J17" t="n">
+        <v>64080</v>
+      </c>
+      <c r="K17" t="n">
+        <v>-52073</v>
+      </c>
+      <c r="L17" t="n">
+        <v>-1.15</v>
+      </c>
+      <c r="M17" t="n">
+        <v>-0.38</v>
+      </c>
+      <c r="N17" t="n">
+        <v>22.81</v>
+      </c>
+      <c r="O17" t="n">
+        <v>23.81</v>
+      </c>
+      <c r="P17" t="n">
+        <v>21.56</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>13247</v>
+      </c>
+      <c r="R17" t="n">
+        <v>-8195</v>
+      </c>
+      <c r="S17" t="n">
+        <v>-8549</v>
+      </c>
+      <c r="T17" t="n">
+        <v>8635</v>
+      </c>
+      <c r="U17" t="n">
+        <v>4612</v>
+      </c>
+      <c r="V17" t="n">
+        <v>8468</v>
+      </c>
+      <c r="W17" t="n">
+        <v>6096</v>
+      </c>
+      <c r="X17" t="n">
+        <v>28986</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>65823</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>94.45999999999999</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>22272</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>21285</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>7079</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
         <v>44286</v>
       </c>
-      <c r="B17" t="n">
-        <v>87.61</v>
-      </c>
-      <c r="C17" t="n">
-        <v>30.35</v>
-      </c>
-      <c r="D17" t="n">
+      <c r="B18" t="n">
+        <v>87.53</v>
+      </c>
+      <c r="C18" t="n">
+        <v>30.32</v>
+      </c>
+      <c r="D18" t="n">
         <v>3.3</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E18" t="n">
         <v>13350</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F18" t="n">
         <v>36.29</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G18" t="n">
         <v>6.22</v>
       </c>
-      <c r="H17" t="n">
-        <v>832007280</v>
-      </c>
-      <c r="I17" t="n">
+      <c r="H18" t="n">
+        <v>831238590.0000001</v>
+      </c>
+      <c r="I18" t="n">
         <v>11614</v>
       </c>
-      <c r="J17" t="n">
+      <c r="J18" t="n">
         <v>64219</v>
       </c>
-      <c r="K17" t="n">
+      <c r="K18" t="n">
         <v>-52605</v>
       </c>
-      <c r="L17" t="n">
+      <c r="L18" t="n">
         <v>-1.38</v>
       </c>
-      <c r="M17" t="n">
+      <c r="M18" t="n">
         <v>-0.39</v>
       </c>
-      <c r="N17" t="n">
-        <v>23.13</v>
-      </c>
-      <c r="O17" t="n">
+      <c r="N18" t="n">
+        <v>23.11</v>
+      </c>
+      <c r="O18" t="n">
         <v>20.52</v>
       </c>
-      <c r="P17" t="n">
+      <c r="P18" t="n">
         <v>18.63</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="Q18" t="n">
         <v>12242</v>
       </c>
-      <c r="R17" t="n">
+      <c r="R18" t="n">
         <v>-4874</v>
       </c>
-      <c r="S17" t="n">
+      <c r="S18" t="n">
         <v>-5185</v>
       </c>
-      <c r="T17" t="n">
+      <c r="T18" t="n">
         <v>7970</v>
       </c>
-      <c r="U17" t="n">
+      <c r="U18" t="n">
         <v>4272</v>
       </c>
-      <c r="V17" t="n">
+      <c r="V18" t="n">
         <v>7803</v>
       </c>
-      <c r="W17" t="n">
+      <c r="W18" t="n">
         <v>5197</v>
       </c>
-      <c r="X17" t="n">
+      <c r="X18" t="n">
         <v>26240</v>
       </c>
-      <c r="Y17" t="n">
+      <c r="Y18" t="n">
         <v>64605</v>
       </c>
-      <c r="Z17" t="n">
+      <c r="Z18" t="n">
         <v>100.35</v>
       </c>
-      <c r="AA17" t="n">
+      <c r="AA18" t="n">
         <v>18146</v>
       </c>
-      <c r="AB17" t="n">
+      <c r="AB18" t="n">
         <v>17092</v>
       </c>
-      <c r="AC17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE17" t="n">
+      <c r="AC18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE18" t="n">
         <v>3939</v>
       </c>
     </row>

</xml_diff>